<commit_message>
Updated to include Jump, Branch, MemRead
</commit_message>
<xml_diff>
--- a/Proj1_control_signals.xlsx
+++ b/Proj1_control_signals.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="90">
   <si>
     <t xml:space="preserve">Instruction</t>
   </si>
@@ -90,6 +90,15 @@
   </si>
   <si>
     <t xml:space="preserve">RegDst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jump</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MemRead</t>
   </si>
   <si>
     <t xml:space="preserve">Note: these are example control signals from the text and your skeleton code; you will need to add more control signals; you may rename any control signals, except those given in the skeleton code.</t>
@@ -490,7 +499,7 @@
       <c r="N1" s="3"/>
       <c r="O1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -512,25 +521,34 @@
       <c r="I2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="0" t="s">
         <v>10</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D3" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
@@ -544,26 +562,35 @@
       <c r="I3" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>15</v>
+      <c r="J3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="F4" s="1" t="n">
         <v>0</v>
       </c>
@@ -576,23 +603,31 @@
       <c r="I4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="0"/>
+      <c r="J4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>0</v>
@@ -604,24 +639,33 @@
         <v>1</v>
       </c>
       <c r="I5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>0</v>
@@ -634,23 +678,32 @@
       </c>
       <c r="I6" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>0</v>
@@ -663,23 +716,32 @@
       </c>
       <c r="I7" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>0</v>
@@ -691,24 +753,33 @@
         <v>1</v>
       </c>
       <c r="I8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>0</v>
@@ -720,24 +791,33 @@
         <v>1</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="J9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>1</v>
@@ -750,23 +830,32 @@
       </c>
       <c r="I10" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="J10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>0</v>
@@ -779,23 +868,32 @@
       </c>
       <c r="I11" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>0</v>
@@ -808,23 +906,32 @@
       </c>
       <c r="I12" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F13" s="1" t="n">
         <v>0</v>
@@ -836,24 +943,33 @@
         <v>1</v>
       </c>
       <c r="I13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D14" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>0</v>
@@ -866,23 +982,32 @@
       </c>
       <c r="I14" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>0</v>
@@ -894,24 +1019,33 @@
         <v>1</v>
       </c>
       <c r="I15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D16" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>0</v>
@@ -924,23 +1058,32 @@
       </c>
       <c r="I16" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F17" s="1" t="n">
         <v>0</v>
@@ -952,24 +1095,33 @@
         <v>1</v>
       </c>
       <c r="I17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F18" s="1" t="n">
         <v>0</v>
@@ -982,23 +1134,32 @@
       </c>
       <c r="I18" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F19" s="1" t="n">
         <v>0</v>
@@ -1011,23 +1172,32 @@
       </c>
       <c r="I19" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D20" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F20" s="1" t="n">
         <v>0</v>
@@ -1040,52 +1210,70 @@
       </c>
       <c r="I20" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D21" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>32</v>
+      <c r="J21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D22" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F22" s="1" t="n">
         <v>0</v>
@@ -1098,23 +1286,32 @@
       </c>
       <c r="I22" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D23" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F23" s="1" t="n">
         <v>0</v>
@@ -1127,23 +1324,32 @@
       </c>
       <c r="I23" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D24" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F24" s="1" t="n">
         <v>0</v>
@@ -1155,24 +1361,33 @@
         <v>0</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="J24" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D25" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F25" s="1" t="n">
         <v>0</v>
@@ -1184,24 +1399,33 @@
         <v>0</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="J25" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F26" s="1" t="n">
         <v>0</v>
@@ -1213,24 +1437,33 @@
         <v>0</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="J26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F27" s="1" t="n">
         <v>0</v>
@@ -1242,25 +1475,34 @@
         <v>1</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="J27" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="F28" s="1" t="n">
         <v>0</v>
       </c>
@@ -1271,24 +1513,33 @@
         <v>0</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="J28" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="16" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D29" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F29" s="1" t="n">
         <v>1</v>
@@ -1301,23 +1552,32 @@
       </c>
       <c r="I29" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="J29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D30" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F30" s="1" t="n">
         <v>1</v>
@@ -1330,23 +1590,32 @@
       </c>
       <c r="I30" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="J30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D31" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F31" s="1" t="n">
         <v>1</v>
@@ -1359,23 +1628,32 @@
       </c>
       <c r="I31" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="J31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D32" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F32" s="1" t="n">
         <v>1</v>
@@ -1388,23 +1666,32 @@
       </c>
       <c r="I32" s="1" t="n">
         <v>0</v>
+      </c>
+      <c r="J32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D33" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="F33" s="1" t="n">
         <v>0</v>
@@ -1417,23 +1704,32 @@
       </c>
       <c r="I33" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D34" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F34" s="1" t="n">
         <v>0</v>
@@ -1446,23 +1742,32 @@
       </c>
       <c r="I34" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D35" s="1" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F35" s="1" t="n">
         <v>0</v>
@@ -1475,6 +1780,15 @@
       </c>
       <c r="I35" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="J35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>